<commit_message>
Regenerate the 16 Current TAPPs xlsx with the fixed exporter
Styling only. Every one of these was exported by the version of
tapp_to_xlsx.py that counted Purpose as a mode flag, so each carried
Purpose at MODE_COL_WIDTH (13 characters) with centre alignment -- a
13-character column holding a full sentence.

Purpose is now 48 characters wide and top-aligned, and Y/N shading is
confined to the real mode columns. Mode counts now match the documented
table: EPMA 4, LA family 3, Lab-XCT 2, SEM_Composition 4, SEM_FIBSEM 2,
SEM_Imaging 5, SEM 11, TEM 3, Solution Q/SF/MC 0.

No CSV was read for content or written -- the source of truth is unchanged,
and row counts and the Legends sheet are identical to the previous export.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Current TAPPs/EPMA_TAPP_v60.xlsx
+++ b/Current TAPPs/EPMA_TAPP_v60.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAPP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legends" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TAPP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legends" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -543,7 +543,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
@@ -611,7 +611,7 @@
           <t>Keyed By</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
@@ -871,7 +871,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="1" t="n"/>
       <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1011,7 +1011,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="1" t="n"/>
       <c r="K4" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1151,7 +1151,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="J5" s="1" t="n"/>
       <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1291,7 +1291,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="1" t="n"/>
       <c r="K6" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1431,7 +1431,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="1" t="n"/>
       <c r="K7" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1523,7 +1523,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="1" t="n"/>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1615,7 +1615,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n"/>
+      <c r="J9" s="1" t="n"/>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1707,7 +1707,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="1" t="n"/>
       <c r="K10" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1847,7 +1847,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="1" t="inlineStr">
         <is>
           <t>Encourages formal procedure registration and ensures traceability.</t>
         </is>
@@ -1939,7 +1939,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="1" t="inlineStr">
         <is>
           <t>The analysis record corresponds to one session, which may cover several samples, and this is the link back to the raw instrument files.</t>
         </is>
@@ -2027,7 +2027,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n"/>
+      <c r="J13" s="1" t="n"/>
       <c r="K13" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2167,7 +2167,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n"/>
+      <c r="J14" s="1" t="n"/>
       <c r="K14" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2259,7 +2259,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n"/>
+      <c r="J15" s="1" t="n"/>
       <c r="K15" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2351,7 +2351,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n"/>
+      <c r="J16" s="1" t="n"/>
       <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2443,7 +2443,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J17" s="2" t="n"/>
+      <c r="J17" s="1" t="n"/>
       <c r="K17" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2583,7 +2583,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J18" s="2" t="n"/>
+      <c r="J18" s="1" t="n"/>
       <c r="K18" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2723,7 +2723,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J19" s="1" t="inlineStr">
         <is>
           <t>Provides a stable, citable link to the companion method independent of whether a dataset has been deposited.</t>
         </is>
@@ -2819,7 +2819,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n"/>
+      <c r="J20" s="1" t="n"/>
       <c r="K20" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3024,7 +3024,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J23" s="1" t="inlineStr">
         <is>
           <t>Used for discoverability and procedure matching, and because the material type constrains sample preparation, calibration and matrix-matching requirements.</t>
         </is>
@@ -3168,7 +3168,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n"/>
+      <c r="J24" s="1" t="n"/>
       <c r="K24" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3308,7 +3308,7 @@
           <t>defines: sample</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J25" s="1" t="inlineStr">
         <is>
           <t>The analysis record corresponds to one session and may cover several samples.</t>
         </is>
@@ -3452,7 +3452,7 @@
           <t>defines: sampling unit</t>
         </is>
       </c>
-      <c r="J26" s="2" t="n"/>
+      <c r="J26" s="1" t="n"/>
       <c r="K26" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3536,7 +3536,7 @@
           <t>sample</t>
         </is>
       </c>
-      <c r="J27" s="2" t="n"/>
+      <c r="J27" s="1" t="n"/>
       <c r="K27" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3636,7 +3636,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J28" s="2" t="n"/>
+      <c r="J28" s="1" t="n"/>
       <c r="K28" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3716,7 +3716,7 @@
           <t>sample</t>
         </is>
       </c>
-      <c r="J29" s="2" t="n"/>
+      <c r="J29" s="1" t="n"/>
       <c r="K29" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3913,7 +3913,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J32" s="1" t="inlineStr">
         <is>
           <t>Recording it as a controlled value lets procedures be found by vendor.</t>
         </is>
@@ -4057,7 +4057,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J33" s="2" t="n"/>
+      <c r="J33" s="1" t="n"/>
       <c r="K33" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4193,7 +4193,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J34" s="2" t="n"/>
+      <c r="J34" s="1" t="n"/>
       <c r="K34" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4333,7 +4333,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J35" s="2" t="n"/>
+      <c r="J35" s="1" t="n"/>
       <c r="K35" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4473,7 +4473,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J36" s="2" t="n"/>
+      <c r="J36" s="1" t="n"/>
       <c r="K36" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4609,7 +4609,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n"/>
+      <c r="J37" s="1" t="n"/>
       <c r="K37" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -4745,7 +4745,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J38" s="2" t="n"/>
+      <c r="J38" s="1" t="n"/>
       <c r="K38" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4998,7 +4998,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="J41" s="1" t="inlineStr">
         <is>
           <t>Serves as the procedure-level declaration of measurement type, distinct from the mode flag columns, which state per-field applicability. Ensures every procedure record is self-describing and comparable across the library.</t>
         </is>
@@ -5082,7 +5082,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="J42" s="2" t="n"/>
+      <c r="J42" s="1" t="n"/>
       <c r="K42" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5218,7 +5218,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J43" s="2" t="n"/>
+      <c r="J43" s="1" t="n"/>
       <c r="K43" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5354,7 +5354,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="J44" s="2" t="n"/>
+      <c r="J44" s="1" t="n"/>
       <c r="K44" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5490,7 +5490,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="J45" s="2" t="n"/>
+      <c r="J45" s="1" t="n"/>
       <c r="K45" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5626,7 +5626,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J46" s="1" t="inlineStr">
         <is>
           <t>Averages over a coarse-grained or beam-sensitive phase by distributing dose across a larger area.</t>
         </is>
@@ -5766,7 +5766,7 @@
           <t>sample &gt; sampling unit</t>
         </is>
       </c>
-      <c r="J47" s="2" t="n"/>
+      <c r="J47" s="1" t="n"/>
       <c r="K47" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -5902,7 +5902,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J48" s="2" t="n"/>
+      <c r="J48" s="1" t="n"/>
       <c r="K48" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -6042,7 +6042,7 @@
           <t>defines: analyte</t>
         </is>
       </c>
-      <c r="J49" s="2" t="n"/>
+      <c r="J49" s="1" t="n"/>
       <c r="K49" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -6182,7 +6182,7 @@
           <t>defines: reported property</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="J50" s="1" t="inlineStr">
         <is>
           <t>A procedure may acquire many channels and report a small number of derived quantities; without this field a data consumer cannot tell which.</t>
         </is>
@@ -6266,7 +6266,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J51" s="2" t="n"/>
+      <c r="J51" s="1" t="n"/>
       <c r="K51" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -6402,7 +6402,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="J52" s="1" t="inlineStr">
         <is>
           <t>Line choice affects sensitivity, matrix correction accuracy, and susceptibility to peak overlap and spectral interference.</t>
         </is>
@@ -6542,7 +6542,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="J53" s="1" t="inlineStr">
         <is>
           <t>Crystal choice determines the detectable wavelength range and dispersion.</t>
         </is>
@@ -6682,7 +6682,7 @@
           <t>defines: channel per analyte</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="J54" s="1" t="inlineStr">
         <is>
           <t>Different spectrometers may have different crystal configurations.</t>
         </is>
@@ -6822,7 +6822,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="J55" s="1" t="inlineStr">
         <is>
           <t>Relevant for minimizing beam damage (volatile elements measured first) and for sequential multi-channel setups.</t>
         </is>
@@ -6962,7 +6962,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="J56" s="1" t="inlineStr">
         <is>
           <t>Affects sensitivity and count rate linearity.</t>
         </is>
@@ -7102,7 +7102,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J57" s="2" t="n"/>
+      <c r="J57" s="1" t="n"/>
       <c r="K57" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -7238,7 +7238,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J58" s="2" t="n"/>
+      <c r="J58" s="1" t="n"/>
       <c r="K58" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -7374,7 +7374,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J59" s="2" t="n"/>
+      <c r="J59" s="1" t="n"/>
       <c r="K59" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -7510,7 +7510,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J60" s="2" t="n"/>
+      <c r="J60" s="1" t="n"/>
       <c r="K60" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -7646,7 +7646,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J61" s="2" t="n"/>
+      <c r="J61" s="1" t="n"/>
       <c r="K61" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -7782,7 +7782,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="J62" s="1" t="inlineStr">
         <is>
           <t>Particularly important when a procedure includes linescans as a distinct acquisition approach not fully captured by the mode flag columns.</t>
         </is>
@@ -7866,7 +7866,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J63" s="2" t="n"/>
+      <c r="J63" s="1" t="n"/>
       <c r="K63" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -8002,7 +8002,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J64" s="2" t="n"/>
+      <c r="J64" s="1" t="n"/>
       <c r="K64" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -8138,7 +8138,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J65" s="2" t="n"/>
+      <c r="J65" s="1" t="n"/>
       <c r="K65" s="13" t="inlineStr">
         <is>
           <t>N</t>
@@ -8274,7 +8274,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="J66" s="1" t="inlineStr">
         <is>
           <t>Based on the sample feature or region of interest, so it is chosen to cover the target.</t>
         </is>
@@ -8414,7 +8414,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="J67" s="1" t="inlineStr">
         <is>
           <t>Stage scan preserves beam geometry and spot size across the full map but is slower; beam scan is faster but may introduce geometric distortion at large deflections.</t>
         </is>
@@ -8667,7 +8667,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J70" s="2" t="n"/>
+      <c r="J70" s="1" t="n"/>
       <c r="K70" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8803,7 +8803,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr">
+      <c r="J71" s="1" t="inlineStr">
         <is>
           <t>MAC database choice affects accuracy particularly for light elements (B, C, N, O, F, Na).</t>
         </is>
@@ -8943,7 +8943,7 @@
           <t>channel</t>
         </is>
       </c>
-      <c r="J72" s="2" t="n"/>
+      <c r="J72" s="1" t="n"/>
       <c r="K72" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9079,7 +9079,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="J73" s="1" t="inlineStr">
         <is>
           <t>Most commonly applied in point analysis; uncommon for X-ray mapping.</t>
         </is>
@@ -9219,7 +9219,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J74" s="2" t="n"/>
+      <c r="J74" s="1" t="n"/>
       <c r="K74" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9355,7 +9355,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J75" s="2" t="n"/>
+      <c r="J75" s="1" t="n"/>
       <c r="K75" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9491,7 +9491,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
+      <c r="J76" s="1" t="inlineStr">
         <is>
           <t>Dead time errors are most significant for major elements with high count rates (e.g., Si, Fe, Ca).</t>
         </is>
@@ -9631,7 +9631,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J77" s="2" t="n"/>
+      <c r="J77" s="1" t="n"/>
       <c r="K77" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9767,7 +9767,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J78" s="2" t="n"/>
+      <c r="J78" s="1" t="n"/>
       <c r="K78" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9907,7 +9907,7 @@
           <t>reported property</t>
         </is>
       </c>
-      <c r="J79" s="2" t="n"/>
+      <c r="J79" s="1" t="n"/>
       <c r="K79" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10043,7 +10043,7 @@
           <t>reported property</t>
         </is>
       </c>
-      <c r="J80" s="2" t="n"/>
+      <c r="J80" s="1" t="n"/>
       <c r="K80" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10123,7 +10123,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
+      <c r="J81" s="1" t="inlineStr">
         <is>
           <t>Follows the criterion-versus-measurement split the library applies wherever a procedure sets a threshold and an analysis reports a value against it.</t>
         </is>
@@ -10207,7 +10207,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
+      <c r="J82" s="1" t="inlineStr">
         <is>
           <t>Criteria and outcome are combined in one field because neither is interpretable without the other, following the precision/accuracy precedent.</t>
         </is>
@@ -10295,7 +10295,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J83" s="2" t="n"/>
+      <c r="J83" s="1" t="n"/>
       <c r="K83" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10492,7 +10492,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
+      <c r="J86" s="1" t="inlineStr">
         <is>
           <t>Results calibrated against different published values for the same material are not directly comparable.</t>
         </is>
@@ -10636,7 +10636,7 @@
           <t>defines: standard</t>
         </is>
       </c>
-      <c r="J87" s="2" t="n"/>
+      <c r="J87" s="1" t="n"/>
       <c r="K87" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10772,7 +10772,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J88" s="2" t="n"/>
+      <c r="J88" s="1" t="n"/>
       <c r="K88" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10908,7 +10908,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J89" s="2" t="n"/>
+      <c r="J89" s="1" t="n"/>
       <c r="K89" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11000,7 +11000,7 @@
           <t>analyte</t>
         </is>
       </c>
-      <c r="J90" s="2" t="n"/>
+      <c r="J90" s="1" t="n"/>
       <c r="K90" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11092,7 +11092,7 @@
           <t>reported property</t>
         </is>
       </c>
-      <c r="J91" s="2" t="n"/>
+      <c r="J91" s="1" t="n"/>
       <c r="K91" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11232,7 +11232,7 @@
           <t>reported property</t>
         </is>
       </c>
-      <c r="J92" s="2" t="n"/>
+      <c r="J92" s="1" t="n"/>
       <c r="K92" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11368,7 +11368,7 @@
           <t>standard x reported property</t>
         </is>
       </c>
-      <c r="J93" s="2" t="n"/>
+      <c r="J93" s="1" t="n"/>
       <c r="K93" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11504,7 +11504,7 @@
           <t>standard x reported property</t>
         </is>
       </c>
-      <c r="J94" s="2" t="n"/>
+      <c r="J94" s="1" t="n"/>
       <c r="K94" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11644,7 +11644,7 @@
           <t>sample &gt; sampling unit x reported property</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr">
+      <c r="J95" s="1" t="inlineStr">
         <is>
           <t>Where a procedure reports both, agreement indicates the measurement is shot-noise limited, and a larger observed scatter indicates a further source of variance.</t>
         </is>
@@ -11784,7 +11784,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J96" s="2" t="inlineStr">
+      <c r="J96" s="1" t="inlineStr">
         <is>
           <t>Values above ~40% indicate excessive count rate and may degrade spectral quality and quantitative accuracy. EDS dead time correction is managed automatically by the detector electronics.</t>
         </is>
@@ -11924,7 +11924,7 @@
           <t>reported property</t>
         </is>
       </c>
-      <c r="J97" s="2" t="inlineStr">
+      <c r="J97" s="1" t="inlineStr">
         <is>
           <t>Answers whether a reported aggregate is defensible as a single population. The value cannot be known before the analysis.</t>
         </is>
@@ -12012,7 +12012,7 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="J98" s="2" t="n"/>
+      <c r="J98" s="1" t="n"/>
       <c r="K98" s="8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -12117,7 +12117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12241,7 +12241,7 @@
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>EDS Point Analysis</t>
         </is>
       </c>
       <c r="B9" s="1" t="n"/>
@@ -12249,7 +12249,7 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>EDS Point Analysis</t>
+          <t>EDS Mapping</t>
         </is>
       </c>
       <c r="B10" s="1" t="n"/>
@@ -12257,7 +12257,7 @@
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>EDS Mapping</t>
+          <t>WDS Point Analysis</t>
         </is>
       </c>
       <c r="B11" s="1" t="n"/>
@@ -12265,298 +12265,290 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>WDS Point Analysis</t>
+          <t>WDS Mapping</t>
         </is>
       </c>
       <c r="B12" s="1" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>WDS Mapping</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="n"/>
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>This field applies to this analytical mode and should be reported.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>This field applies to this analytical mode and should be reported.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
           <t>This field does not apply to this analytical mode.</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>What to enter</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>Data Type</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>What to enter</t>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Controlled list</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Choose one of the values listed in "Example / Allowed Content". The list is CLOSED — it is meant to cover every case. If your value genuinely is not there, that is a gap in the list worth reporting, not a reason to write your own.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Controlled list</t>
+          <t>Controlled list / Text</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Choose one of the values listed in "Example / Allowed Content". The list is CLOSED — it is meant to cover every case. If your value genuinely is not there, that is a gap in the list worth reporting, not a reason to write your own.</t>
+          <t>Choose a listed value AND qualify it in the same cell — the detail is expected, not optional. Typically what was corrected, which analytes or phases it applied to, the method or equation used, or the source it came from. An answer the list cannot express is also valid here.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Controlled list / Text</t>
+          <t>Numeric (unit)</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>Choose a listed value AND qualify it in the same cell — the detail is expected, not optional. Typically what was corrected, which analytes or phases it applied to, the method or equation used, or the source it came from. An answer the list cannot express is also valid here.</t>
+          <t>A number in the unit named in brackets. Enter the number only — the unit is fixed by the field.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Numeric (unit)</t>
+          <t>Numeric + unit</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>A number in the unit named in brackets. Enter the number only — the unit is fixed by the field.</t>
+          <t>A number AND its unit, because the unit varies between procedures. Write both, e.g. '50 us' or '0.5 s'.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Numeric + unit</t>
+          <t>Text (free)</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>A number AND its unit, because the unit varies between procedures. Write both, e.g. '50 us' or '0.5 s'.</t>
+          <t>Free text. No controlled vocabulary applies.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
-          <t>Text (free)</t>
+          <t>N/A | None</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>Free text. No controlled vocabulary applies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>N/A | None</t>
-        </is>
-      </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
           <t>Offered by every controlled list. "N/A" means the field does not apply to this procedure; "None" means it applies but nothing was used. Prefer either over leaving the cell blank.</t>
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Keyed By (Rule 7)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>What the field's value repeats over</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Keyed By (Rule 7)</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>What the field's value repeats over</t>
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Scalar — one value per procedure or analysis. The default.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>(none)</t>
+          <t>analyte</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Scalar — one value per procedure or analysis. The default.</t>
+          <t>One value per chemical species determined, at whatever granularity the procedure determines it.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="inlineStr">
         <is>
-          <t>analyte</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>One value per chemical species determined, at whatever granularity the procedure determines it.</t>
+          <t>One value per position on the instrument's selection axis — the address, not the signal. Mass, cup, line + crystal, energy-loss edge, wavenumber.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>defines: analyte</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>One value per position on the instrument's selection axis — the address, not the signal. Mass, cup, line + crystal, energy-loss edge, wavenumber.</t>
+          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per chemical species determined, at whatever granularity the procedure determines it.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="20" t="inlineStr">
         <is>
-          <t>defines: analyte</t>
+          <t>defines: channel per analyte</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per chemical species determined, at whatever granularity the procedure determines it.</t>
+          <t>ENUMERATES the channel domain — the header of the child table, not a column in it — and does so once per analyte. One value per position on the instrument's selection axis — the address, not the signal. Mass, cup, line + crystal, energy-loss edge, wavenumber. One value per chemical species determined, at whatever granularity the procedure determines it.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>defines: channel per analyte</t>
+          <t>defines: reported property</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>ENUMERATES the channel domain — the header of the child table, not a column in it — and does so once per analyte. One value per position on the instrument's selection axis — the address, not the signal. Mass, cup, line + crystal, energy-loss edge, wavenumber. One value per chemical species determined, at whatever granularity the procedure determines it.</t>
+          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="20" t="inlineStr">
         <is>
-          <t>defines: reported property</t>
+          <t>defines: sample</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
+          <t xml:space="preserve">ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="20" t="inlineStr">
         <is>
-          <t>defines: sample</t>
+          <t>defines: sampling unit</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. </t>
+          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t>defines: sampling unit</t>
+          <t>defines: standard</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume.</t>
+          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per reference material or reference database entry.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t>defines: standard</t>
+          <t>reported property</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>ENUMERATES the key domain rather than being keyed by it — the header of the child table, not a column in it. One value per reference material or reference database entry.</t>
+          <t>One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>reported property</t>
-        </is>
-      </c>
-      <c r="B37" s="1" t="inlineStr">
-        <is>
-          <t>One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
-        </is>
-      </c>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
         <is>
-          <t>sample</t>
-        </is>
-      </c>
-      <c r="B38" s="1" t="inlineStr"/>
+          <t>sample &gt; sampling unit</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Nested — sampling unit exists only within sample. One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="20" t="inlineStr">
         <is>
-          <t>sample &gt; sampling unit</t>
+          <t>sample &gt; sampling unit x reported property</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Nested — sampling unit exists only within sample. One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume.</t>
+          <t>Cross-product, read as "for each sample, one value per reported property". One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume. + One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
         <is>
-          <t>sample &gt; sampling unit x reported property</t>
+          <t>standard x reported property</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
-        <is>
-          <t>Cross-product, read as "for each sample, one value per reported property". One value per subdivision of the physical sample that carries its own row — grain, spot, aliquot, phase, sub-volume. + One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>standard x reported property</t>
-        </is>
-      </c>
-      <c r="B41" s="1" t="inlineStr">
         <is>
           <t>Cross-product, read as "for each standard, one value per reported property". One value per reference material or reference database entry. + One value per reported quantity or nominal property, at any point in the chain — ratios and dates alike, plus their uncertainties.</t>
         </is>

</xml_diff>